<commit_message>
respaldo automático 2026-08-03 14:39:09
</commit_message>
<xml_diff>
--- a/nexus/tag-web/cache/tagtico-tags.xlsx
+++ b/nexus/tag-web/cache/tagtico-tags.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\DESKTOP-NIOGT1I\Users\Tagtico2\OneDrive\Escritorio\Rendiciones Tag\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tagtico2\OneDrive\Escritorio\Rendiciones Tag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3627DC09-E2D3-4CFF-A76F-54C395D18F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47E0B91D-7333-48D2-B7FE-A78674AB9450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,19 +24,31 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AÑO 2023'!$A$1:$G$217</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AÑO 2024'!$A$1:$G$231</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AÑO 2025'!$A$1:$G$268</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'AÑO 2026'!$A$1:$G$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'AÑO 2026'!$A$1:$G$159</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4408" uniqueCount="1130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4521" uniqueCount="1146">
   <si>
     <t>MONTO</t>
   </si>
@@ -3426,6 +3438,54 @@
   </si>
   <si>
     <t>AGROCOMERCIAL 4 SOLES</t>
+  </si>
+  <si>
+    <t>TKXY30</t>
+  </si>
+  <si>
+    <t>SALVADOR MANZOR</t>
+  </si>
+  <si>
+    <t>SEBASTIAN IRARRAZAVAL</t>
+  </si>
+  <si>
+    <t>HLDC70</t>
+  </si>
+  <si>
+    <t>MATIAS PEREZ</t>
+  </si>
+  <si>
+    <t>SZPV13</t>
+  </si>
+  <si>
+    <t>JAIME SEPULVEDA</t>
+  </si>
+  <si>
+    <t>MAURICIO JARA</t>
+  </si>
+  <si>
+    <t>VON SPA</t>
+  </si>
+  <si>
+    <t>INGENIERIA Y CONSTRUCCION</t>
+  </si>
+  <si>
+    <t>FRANCO ANGULO</t>
+  </si>
+  <si>
+    <t>YICHUAN SHAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUIS MARQUES SILVA DE BALBOA </t>
+  </si>
+  <si>
+    <t>PAULA CARTER</t>
+  </si>
+  <si>
+    <t>RICARDO MAYORGA</t>
+  </si>
+  <si>
+    <t>WINDMADE</t>
   </si>
 </sst>
 </file>
@@ -21895,7 +21955,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19B3CF06-6FB5-4DC6-B5B9-AD7C386B2CA3}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G161"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -24648,7 +24708,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
         <v>12000</v>
       </c>
@@ -24668,10 +24728,10 @@
         <v>755</v>
       </c>
       <c r="G125" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
         <v>12000</v>
       </c>
@@ -24691,10 +24751,10 @@
         <v>34</v>
       </c>
       <c r="G126" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
         <v>12000</v>
       </c>
@@ -24714,10 +24774,10 @@
         <v>397</v>
       </c>
       <c r="G127" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
         <v>12000</v>
       </c>
@@ -24737,10 +24797,10 @@
         <v>218</v>
       </c>
       <c r="G128" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
         <v>12000</v>
       </c>
@@ -24760,10 +24820,10 @@
         <v>21</v>
       </c>
       <c r="G129" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
         <v>6300</v>
       </c>
@@ -24777,10 +24837,10 @@
       </c>
       <c r="F130" s="5"/>
       <c r="G130" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
         <v>12000</v>
       </c>
@@ -24800,10 +24860,10 @@
         <v>136</v>
       </c>
       <c r="G131" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
         <v>12000</v>
       </c>
@@ -24823,10 +24883,10 @@
         <v>463</v>
       </c>
       <c r="G132" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
         <v>12000</v>
       </c>
@@ -24846,10 +24906,10 @@
         <v>46</v>
       </c>
       <c r="G133" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
         <v>12000</v>
       </c>
@@ -24869,10 +24929,10 @@
         <v>522</v>
       </c>
       <c r="G134" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
         <v>12000</v>
       </c>
@@ -24892,10 +24952,10 @@
         <v>34</v>
       </c>
       <c r="G135" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
         <v>12000</v>
       </c>
@@ -24915,10 +24975,10 @@
         <v>136</v>
       </c>
       <c r="G136" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
         <v>12000</v>
       </c>
@@ -24938,10 +24998,10 @@
         <v>136</v>
       </c>
       <c r="G137" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
         <v>6300</v>
       </c>
@@ -24955,10 +25015,10 @@
       </c>
       <c r="F138" s="5"/>
       <c r="G138" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
         <v>12000</v>
       </c>
@@ -24978,10 +25038,10 @@
         <v>46</v>
       </c>
       <c r="G139" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
         <v>12000</v>
       </c>
@@ -25001,10 +25061,10 @@
         <v>46</v>
       </c>
       <c r="G140" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
         <v>12000</v>
       </c>
@@ -25024,10 +25084,10 @@
         <v>218</v>
       </c>
       <c r="G141" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
         <v>12000</v>
       </c>
@@ -25047,10 +25107,10 @@
         <v>375</v>
       </c>
       <c r="G142" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
         <v>12000</v>
       </c>
@@ -25070,10 +25130,10 @@
         <v>166</v>
       </c>
       <c r="G143" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
         <v>12000</v>
       </c>
@@ -25093,10 +25153,10 @@
         <v>149</v>
       </c>
       <c r="G144" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
         <v>12000</v>
       </c>
@@ -25116,10 +25176,10 @@
         <v>81</v>
       </c>
       <c r="G145" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
         <v>12000</v>
       </c>
@@ -25139,10 +25199,10 @@
         <v>375</v>
       </c>
       <c r="G146" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
         <v>12000</v>
       </c>
@@ -25162,10 +25222,10 @@
         <v>375</v>
       </c>
       <c r="G147" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>12000</v>
       </c>
@@ -25185,10 +25245,10 @@
         <v>149</v>
       </c>
       <c r="G148" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
         <v>12000</v>
       </c>
@@ -25208,10 +25268,10 @@
         <v>34</v>
       </c>
       <c r="G149" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>12000</v>
       </c>
@@ -25231,10 +25291,10 @@
         <v>375</v>
       </c>
       <c r="G150" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
         <v>12000</v>
       </c>
@@ -25254,10 +25314,10 @@
         <v>145</v>
       </c>
       <c r="G151" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
         <v>12000</v>
       </c>
@@ -25277,10 +25337,10 @@
         <v>46</v>
       </c>
       <c r="G152" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="4">
         <v>12000</v>
       </c>
@@ -25300,10 +25360,10 @@
         <v>136</v>
       </c>
       <c r="G153" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="4">
         <v>12000</v>
       </c>
@@ -25323,10 +25383,10 @@
         <v>31</v>
       </c>
       <c r="G154" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="4">
         <v>6300</v>
       </c>
@@ -25340,10 +25400,10 @@
       </c>
       <c r="F155" s="5"/>
       <c r="G155" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="4">
         <v>12000</v>
       </c>
@@ -25363,10 +25423,10 @@
         <v>57</v>
       </c>
       <c r="G156" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="4">
         <v>12000</v>
       </c>
@@ -25386,44 +25446,613 @@
         <v>180</v>
       </c>
       <c r="G157" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A158" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B158" s="5" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C158" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E158" s="6">
+        <v>46204</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="G158" s="7" t="s">
         <v>1076</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A158" s="4"/>
-      <c r="B158" s="5"/>
-      <c r="C158" s="5"/>
-      <c r="D158" s="5"/>
-      <c r="E158" s="6"/>
-      <c r="F158" s="5"/>
-      <c r="G158" s="7"/>
-    </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A159" s="4"/>
-      <c r="B159" s="5"/>
-      <c r="C159" s="5"/>
-      <c r="D159" s="5"/>
-      <c r="E159" s="6"/>
-      <c r="F159" s="5"/>
-      <c r="G159" s="7"/>
-    </row>
-    <row r="160" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A160" s="4"/>
-      <c r="B160" s="5"/>
-      <c r="C160" s="5"/>
-      <c r="D160" s="5"/>
-      <c r="E160" s="6"/>
-      <c r="F160" s="5"/>
-      <c r="G160" s="7"/>
-    </row>
-    <row r="161" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="8">
-        <f>SUBTOTAL(9,A2:A160)</f>
-        <v>378900</v>
+      <c r="A159" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B159" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C159" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E159" s="6">
+        <v>46204</v>
+      </c>
+      <c r="F159" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G159" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A160" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B160" s="5" t="s">
+        <v>912</v>
+      </c>
+      <c r="C160" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E160" s="6">
+        <v>46204</v>
+      </c>
+      <c r="F160" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G160" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A161" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B161" s="5" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C161" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D161" s="5" t="s">
+        <v>1131</v>
+      </c>
+      <c r="E161" s="6">
+        <v>46206</v>
+      </c>
+      <c r="F161" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G161" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B162" s="5" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C162" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D162" s="5" t="s">
+        <v>1132</v>
+      </c>
+      <c r="E162" s="6">
+        <v>46206</v>
+      </c>
+      <c r="F162" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="G162" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" s="4">
+        <v>6000</v>
+      </c>
+      <c r="B163" s="5"/>
+      <c r="C163" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D163" s="5"/>
+      <c r="E163" s="6">
+        <v>46209</v>
+      </c>
+      <c r="F163" s="5"/>
+      <c r="G163" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A164" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B164" s="5" t="s">
+        <v>904</v>
+      </c>
+      <c r="C164" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D164" s="5" t="s">
+        <v>1110</v>
+      </c>
+      <c r="E164" s="6">
+        <v>46209</v>
+      </c>
+      <c r="F164" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G164" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A165" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B165" s="5" t="s">
+        <v>1133</v>
+      </c>
+      <c r="C165" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D165" s="5" t="s">
+        <v>1134</v>
+      </c>
+      <c r="E165" s="6">
+        <v>46210</v>
+      </c>
+      <c r="F165" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="G165" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A166" s="4">
+        <v>6000</v>
+      </c>
+      <c r="B166" s="5"/>
+      <c r="C166" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D166" s="5"/>
+      <c r="E166" s="6">
+        <v>46216</v>
+      </c>
+      <c r="F166" s="5"/>
+      <c r="G166" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A167" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B167" s="5" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C167" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D167" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E167" s="6">
+        <v>46216</v>
+      </c>
+      <c r="F167" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G167" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A168" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B168" s="5" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C168" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D168" s="5" t="s">
+        <v>1136</v>
+      </c>
+      <c r="E168" s="6">
+        <v>46220</v>
+      </c>
+      <c r="F168" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G168" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A169" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B169" s="5" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C169" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D169" s="5" t="s">
+        <v>1137</v>
+      </c>
+      <c r="E169" s="6">
+        <v>46220</v>
+      </c>
+      <c r="F169" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="G169" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A170" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B170" s="5" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C170" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D170" s="5" t="s">
+        <v>1138</v>
+      </c>
+      <c r="E170" s="6">
+        <v>46220</v>
+      </c>
+      <c r="F170" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G170" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A171" s="4">
+        <v>6000</v>
+      </c>
+      <c r="B171" s="5"/>
+      <c r="C171" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D171" s="5"/>
+      <c r="E171" s="6">
+        <v>46223</v>
+      </c>
+      <c r="F171" s="5"/>
+      <c r="G171" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A172" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B172" s="5" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C172" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D172" s="5" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E172" s="6">
+        <v>46223</v>
+      </c>
+      <c r="F172" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G172" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" s="4">
+        <v>10000</v>
+      </c>
+      <c r="B173" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="C173" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D173" s="5" t="s">
+        <v>1142</v>
+      </c>
+      <c r="E173" s="6">
+        <v>46224</v>
+      </c>
+      <c r="F173" s="5" t="s">
+        <v>755</v>
+      </c>
+      <c r="G173" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A174" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B174" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C174" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D174" s="5" t="s">
+        <v>1140</v>
+      </c>
+      <c r="E174" s="6">
+        <v>46224</v>
+      </c>
+      <c r="F174" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G174" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A175" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B175" s="5" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C175" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D175" s="5" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E175" s="6">
+        <v>46224</v>
+      </c>
+      <c r="F175" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G175" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A176" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B176" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="C176" s="5" t="s">
+        <v>660</v>
+      </c>
+      <c r="D176" s="5" t="s">
+        <v>1142</v>
+      </c>
+      <c r="E176" s="6">
+        <v>46226</v>
+      </c>
+      <c r="F176" s="5" t="s">
+        <v>755</v>
+      </c>
+      <c r="G176" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A177" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B177" s="5" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C177" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D177" s="5" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E177" s="6">
+        <v>46227</v>
+      </c>
+      <c r="F177" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G177" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A178" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B178" s="5" t="s">
+        <v>980</v>
+      </c>
+      <c r="C178" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D178" s="5" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E178" s="6">
+        <v>46227</v>
+      </c>
+      <c r="F178" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G178" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A179" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B179" s="5" t="s">
+        <v>967</v>
+      </c>
+      <c r="C179" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D179" s="5" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E179" s="6">
+        <v>46227</v>
+      </c>
+      <c r="F179" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G179" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A180" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B180" s="5" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C180" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D180" s="5" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E180" s="6">
+        <v>46227</v>
+      </c>
+      <c r="F180" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="G180" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A181" s="4">
+        <v>6000</v>
+      </c>
+      <c r="B181" s="5"/>
+      <c r="C181" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D181" s="5"/>
+      <c r="E181" s="6">
+        <v>46230</v>
+      </c>
+      <c r="F181" s="5"/>
+      <c r="G181" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A182" s="4">
+        <v>12000</v>
+      </c>
+      <c r="B182" s="5" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C182" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D182" s="5" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E182" s="6">
+        <v>46231</v>
+      </c>
+      <c r="F182" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="G182" s="7" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A183" s="4"/>
+      <c r="B183" s="5"/>
+      <c r="C183" s="5"/>
+      <c r="D183" s="5"/>
+      <c r="E183" s="6"/>
+      <c r="F183" s="5"/>
+      <c r="G183" s="7"/>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A184" s="4"/>
+      <c r="B184" s="5"/>
+      <c r="C184" s="5"/>
+      <c r="D184" s="5"/>
+      <c r="E184" s="6"/>
+      <c r="F184" s="5"/>
+      <c r="G184" s="7"/>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A185" s="4"/>
+      <c r="B185" s="5"/>
+      <c r="C185" s="5"/>
+      <c r="D185" s="5"/>
+      <c r="E185" s="6"/>
+      <c r="F185" s="5"/>
+      <c r="G185" s="7"/>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A186" s="4"/>
+      <c r="B186" s="5"/>
+      <c r="C186" s="5"/>
+      <c r="D186" s="5"/>
+      <c r="E186" s="6"/>
+      <c r="F186" s="5"/>
+      <c r="G186" s="7"/>
+    </row>
+    <row r="187" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="4"/>
+      <c r="B187" s="5"/>
+      <c r="C187" s="5"/>
+      <c r="D187" s="5"/>
+      <c r="E187" s="6"/>
+      <c r="F187" s="5"/>
+      <c r="G187" s="7"/>
+    </row>
+    <row r="188" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A188" s="8">
+        <f>SUBTOTAL(9,A2:A187)</f>
+        <v>274000</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G125" xr:uid="{19B3CF06-6FB5-4DC6-B5B9-AD7C386B2CA3}">
+  <autoFilter ref="A1:G159" xr:uid="{19B3CF06-6FB5-4DC6-B5B9-AD7C386B2CA3}">
     <filterColumn colId="6">
       <filters>
         <filter val="PENDIENTE"/>

</xml_diff>

<commit_message>
respaldo automático 2026-08-06 14:40:54
</commit_message>
<xml_diff>
--- a/nexus/tag-web/cache/tagtico-tags.xlsx
+++ b/nexus/tag-web/cache/tagtico-tags.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tagtico2\OneDrive\Escritorio\Rendiciones Tag\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\DESKTOP-NIOGT1I\Users\Tagtico2\OneDrive\Escritorio\Rendiciones Tag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47E0B91D-7333-48D2-B7FE-A78674AB9450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3627DC09-E2D3-4CFF-A76F-54C395D18F6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,31 +24,19 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AÑO 2023'!$A$1:$G$217</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'AÑO 2024'!$A$1:$G$231</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AÑO 2025'!$A$1:$G$268</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'AÑO 2026'!$A$1:$G$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'AÑO 2026'!$A$1:$G$125</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4521" uniqueCount="1146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4408" uniqueCount="1130">
   <si>
     <t>MONTO</t>
   </si>
@@ -3438,54 +3426,6 @@
   </si>
   <si>
     <t>AGROCOMERCIAL 4 SOLES</t>
-  </si>
-  <si>
-    <t>TKXY30</t>
-  </si>
-  <si>
-    <t>SALVADOR MANZOR</t>
-  </si>
-  <si>
-    <t>SEBASTIAN IRARRAZAVAL</t>
-  </si>
-  <si>
-    <t>HLDC70</t>
-  </si>
-  <si>
-    <t>MATIAS PEREZ</t>
-  </si>
-  <si>
-    <t>SZPV13</t>
-  </si>
-  <si>
-    <t>JAIME SEPULVEDA</t>
-  </si>
-  <si>
-    <t>MAURICIO JARA</t>
-  </si>
-  <si>
-    <t>VON SPA</t>
-  </si>
-  <si>
-    <t>INGENIERIA Y CONSTRUCCION</t>
-  </si>
-  <si>
-    <t>FRANCO ANGULO</t>
-  </si>
-  <si>
-    <t>YICHUAN SHAD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LUIS MARQUES SILVA DE BALBOA </t>
-  </si>
-  <si>
-    <t>PAULA CARTER</t>
-  </si>
-  <si>
-    <t>RICARDO MAYORGA</t>
-  </si>
-  <si>
-    <t>WINDMADE</t>
   </si>
 </sst>
 </file>
@@ -21955,7 +21895,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19B3CF06-6FB5-4DC6-B5B9-AD7C386B2CA3}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G188"/>
+  <dimension ref="A1:G161"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -24708,7 +24648,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="125" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
         <v>12000</v>
       </c>
@@ -24728,10 +24668,10 @@
         <v>755</v>
       </c>
       <c r="G125" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
         <v>12000</v>
       </c>
@@ -24751,10 +24691,10 @@
         <v>34</v>
       </c>
       <c r="G126" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
         <v>12000</v>
       </c>
@@ -24774,10 +24714,10 @@
         <v>397</v>
       </c>
       <c r="G127" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
         <v>12000</v>
       </c>
@@ -24797,10 +24737,10 @@
         <v>218</v>
       </c>
       <c r="G128" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
         <v>12000</v>
       </c>
@@ -24820,10 +24760,10 @@
         <v>21</v>
       </c>
       <c r="G129" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" s="4">
         <v>6300</v>
       </c>
@@ -24837,10 +24777,10 @@
       </c>
       <c r="F130" s="5"/>
       <c r="G130" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" s="4">
         <v>12000</v>
       </c>
@@ -24860,10 +24800,10 @@
         <v>136</v>
       </c>
       <c r="G131" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
         <v>12000</v>
       </c>
@@ -24883,10 +24823,10 @@
         <v>463</v>
       </c>
       <c r="G132" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
         <v>12000</v>
       </c>
@@ -24906,10 +24846,10 @@
         <v>46</v>
       </c>
       <c r="G133" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" s="4">
         <v>12000</v>
       </c>
@@ -24929,10 +24869,10 @@
         <v>522</v>
       </c>
       <c r="G134" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="135" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" s="4">
         <v>12000</v>
       </c>
@@ -24952,10 +24892,10 @@
         <v>34</v>
       </c>
       <c r="G135" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" s="4">
         <v>12000</v>
       </c>
@@ -24975,10 +24915,10 @@
         <v>136</v>
       </c>
       <c r="G136" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" s="4">
         <v>12000</v>
       </c>
@@ -24998,10 +24938,10 @@
         <v>136</v>
       </c>
       <c r="G137" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="4">
         <v>6300</v>
       </c>
@@ -25015,10 +24955,10 @@
       </c>
       <c r="F138" s="5"/>
       <c r="G138" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="4">
         <v>12000</v>
       </c>
@@ -25038,10 +24978,10 @@
         <v>46</v>
       </c>
       <c r="G139" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="4">
         <v>12000</v>
       </c>
@@ -25061,10 +25001,10 @@
         <v>46</v>
       </c>
       <c r="G140" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="4">
         <v>12000</v>
       </c>
@@ -25084,10 +25024,10 @@
         <v>218</v>
       </c>
       <c r="G141" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="4">
         <v>12000</v>
       </c>
@@ -25107,10 +25047,10 @@
         <v>375</v>
       </c>
       <c r="G142" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="4">
         <v>12000</v>
       </c>
@@ -25130,10 +25070,10 @@
         <v>166</v>
       </c>
       <c r="G143" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144" s="4">
         <v>12000</v>
       </c>
@@ -25153,10 +25093,10 @@
         <v>149</v>
       </c>
       <c r="G144" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
         <v>12000</v>
       </c>
@@ -25176,10 +25116,10 @@
         <v>81</v>
       </c>
       <c r="G145" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
         <v>12000</v>
       </c>
@@ -25199,10 +25139,10 @@
         <v>375</v>
       </c>
       <c r="G146" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
         <v>12000</v>
       </c>
@@ -25222,10 +25162,10 @@
         <v>375</v>
       </c>
       <c r="G147" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>12000</v>
       </c>
@@ -25245,10 +25185,10 @@
         <v>149</v>
       </c>
       <c r="G148" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
         <v>12000</v>
       </c>
@@ -25268,10 +25208,10 @@
         <v>34</v>
       </c>
       <c r="G149" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>12000</v>
       </c>
@@ -25291,10 +25231,10 @@
         <v>375</v>
       </c>
       <c r="G150" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
         <v>12000</v>
       </c>
@@ -25314,10 +25254,10 @@
         <v>145</v>
       </c>
       <c r="G151" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
         <v>12000</v>
       </c>
@@ -25337,10 +25277,10 @@
         <v>46</v>
       </c>
       <c r="G152" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="4">
         <v>12000</v>
       </c>
@@ -25360,10 +25300,10 @@
         <v>136</v>
       </c>
       <c r="G153" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="4">
         <v>12000</v>
       </c>
@@ -25383,10 +25323,10 @@
         <v>31</v>
       </c>
       <c r="G154" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="4">
         <v>6300</v>
       </c>
@@ -25400,10 +25340,10 @@
       </c>
       <c r="F155" s="5"/>
       <c r="G155" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="4">
         <v>12000</v>
       </c>
@@ -25423,10 +25363,10 @@
         <v>57</v>
       </c>
       <c r="G156" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="4">
         <v>12000</v>
       </c>
@@ -25446,613 +25386,44 @@
         <v>180</v>
       </c>
       <c r="G157" s="7" t="s">
-        <v>47</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A158" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B158" s="5" t="s">
-        <v>1130</v>
-      </c>
-      <c r="C158" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="D158" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="E158" s="6">
-        <v>46204</v>
-      </c>
-      <c r="F158" s="5" t="s">
-        <v>463</v>
-      </c>
-      <c r="G158" s="7" t="s">
-        <v>1076</v>
-      </c>
+      <c r="A158" s="4"/>
+      <c r="B158" s="5"/>
+      <c r="C158" s="5"/>
+      <c r="D158" s="5"/>
+      <c r="E158" s="6"/>
+      <c r="F158" s="5"/>
+      <c r="G158" s="7"/>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A159" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B159" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C159" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="D159" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="E159" s="6">
-        <v>46204</v>
-      </c>
-      <c r="F159" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G159" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A160" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B160" s="5" t="s">
-        <v>912</v>
-      </c>
-      <c r="C160" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="D160" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="E160" s="6">
-        <v>46204</v>
-      </c>
-      <c r="F160" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G160" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A161" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B161" s="5" t="s">
-        <v>1122</v>
-      </c>
-      <c r="C161" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D161" s="5" t="s">
-        <v>1131</v>
-      </c>
-      <c r="E161" s="6">
-        <v>46206</v>
-      </c>
-      <c r="F161" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G161" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A162" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B162" s="5" t="s">
-        <v>1074</v>
-      </c>
-      <c r="C162" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D162" s="5" t="s">
-        <v>1132</v>
-      </c>
-      <c r="E162" s="6">
-        <v>46206</v>
-      </c>
-      <c r="F162" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="G162" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A163" s="4">
-        <v>6000</v>
-      </c>
-      <c r="B163" s="5"/>
-      <c r="C163" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D163" s="5"/>
-      <c r="E163" s="6">
-        <v>46209</v>
-      </c>
-      <c r="F163" s="5"/>
-      <c r="G163" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A164" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B164" s="5" t="s">
-        <v>904</v>
-      </c>
-      <c r="C164" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="D164" s="5" t="s">
-        <v>1110</v>
-      </c>
-      <c r="E164" s="6">
-        <v>46209</v>
-      </c>
-      <c r="F164" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G164" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A165" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B165" s="5" t="s">
-        <v>1133</v>
-      </c>
-      <c r="C165" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="D165" s="5" t="s">
-        <v>1134</v>
-      </c>
-      <c r="E165" s="6">
-        <v>46210</v>
-      </c>
-      <c r="F165" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G165" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A166" s="4">
-        <v>6000</v>
-      </c>
-      <c r="B166" s="5"/>
-      <c r="C166" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D166" s="5"/>
-      <c r="E166" s="6">
-        <v>46216</v>
-      </c>
-      <c r="F166" s="5"/>
-      <c r="G166" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A167" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B167" s="5" t="s">
-        <v>1135</v>
-      </c>
-      <c r="C167" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="D167" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="E167" s="6">
-        <v>46216</v>
-      </c>
-      <c r="F167" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G167" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A168" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B168" s="5" t="s">
-        <v>1123</v>
-      </c>
-      <c r="C168" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D168" s="5" t="s">
-        <v>1136</v>
-      </c>
-      <c r="E168" s="6">
-        <v>46220</v>
-      </c>
-      <c r="F168" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="G168" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A169" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B169" s="5" t="s">
-        <v>1120</v>
-      </c>
-      <c r="C169" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D169" s="5" t="s">
-        <v>1137</v>
-      </c>
-      <c r="E169" s="6">
-        <v>46220</v>
-      </c>
-      <c r="F169" s="5" t="s">
-        <v>375</v>
-      </c>
-      <c r="G169" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A170" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B170" s="5" t="s">
-        <v>1135</v>
-      </c>
-      <c r="C170" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D170" s="5" t="s">
-        <v>1138</v>
-      </c>
-      <c r="E170" s="6">
-        <v>46220</v>
-      </c>
-      <c r="F170" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G170" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A171" s="4">
-        <v>6000</v>
-      </c>
-      <c r="B171" s="5"/>
-      <c r="C171" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D171" s="5"/>
-      <c r="E171" s="6">
-        <v>46223</v>
-      </c>
-      <c r="F171" s="5"/>
-      <c r="G171" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A172" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B172" s="5" t="s">
-        <v>1046</v>
-      </c>
-      <c r="C172" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D172" s="5" t="s">
-        <v>1139</v>
-      </c>
-      <c r="E172" s="6">
-        <v>46223</v>
-      </c>
-      <c r="F172" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G172" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A173" s="4">
-        <v>10000</v>
-      </c>
-      <c r="B173" s="5" t="s">
-        <v>761</v>
-      </c>
-      <c r="C173" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D173" s="5" t="s">
-        <v>1142</v>
-      </c>
-      <c r="E173" s="6">
-        <v>46224</v>
-      </c>
-      <c r="F173" s="5" t="s">
-        <v>755</v>
-      </c>
-      <c r="G173" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A174" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B174" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C174" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D174" s="5" t="s">
-        <v>1140</v>
-      </c>
-      <c r="E174" s="6">
-        <v>46224</v>
-      </c>
-      <c r="F174" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G174" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A175" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B175" s="5" t="s">
-        <v>1019</v>
-      </c>
-      <c r="C175" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D175" s="5" t="s">
-        <v>1141</v>
-      </c>
-      <c r="E175" s="6">
-        <v>46224</v>
-      </c>
-      <c r="F175" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="G175" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A176" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B176" s="5" t="s">
-        <v>761</v>
-      </c>
-      <c r="C176" s="5" t="s">
-        <v>660</v>
-      </c>
-      <c r="D176" s="5" t="s">
-        <v>1142</v>
-      </c>
-      <c r="E176" s="6">
-        <v>46226</v>
-      </c>
-      <c r="F176" s="5" t="s">
-        <v>755</v>
-      </c>
-      <c r="G176" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A177" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B177" s="5" t="s">
-        <v>1009</v>
-      </c>
-      <c r="C177" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D177" s="5" t="s">
-        <v>1143</v>
-      </c>
-      <c r="E177" s="6">
-        <v>46227</v>
-      </c>
-      <c r="F177" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G177" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A178" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B178" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="C178" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D178" s="5" t="s">
-        <v>1144</v>
-      </c>
-      <c r="E178" s="6">
-        <v>46227</v>
-      </c>
-      <c r="F178" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G178" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A179" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B179" s="5" t="s">
-        <v>967</v>
-      </c>
-      <c r="C179" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D179" s="5" t="s">
-        <v>1144</v>
-      </c>
-      <c r="E179" s="6">
-        <v>46227</v>
-      </c>
-      <c r="F179" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G179" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A180" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B180" s="5" t="s">
-        <v>1130</v>
-      </c>
-      <c r="C180" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D180" s="5" t="s">
-        <v>1144</v>
-      </c>
-      <c r="E180" s="6">
-        <v>46227</v>
-      </c>
-      <c r="F180" s="5" t="s">
-        <v>463</v>
-      </c>
-      <c r="G180" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A181" s="4">
-        <v>6000</v>
-      </c>
-      <c r="B181" s="5"/>
-      <c r="C181" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D181" s="5"/>
-      <c r="E181" s="6">
-        <v>46230</v>
-      </c>
-      <c r="F181" s="5"/>
-      <c r="G181" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A182" s="4">
-        <v>12000</v>
-      </c>
-      <c r="B182" s="5" t="s">
-        <v>1116</v>
-      </c>
-      <c r="C182" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D182" s="5" t="s">
-        <v>1145</v>
-      </c>
-      <c r="E182" s="6">
-        <v>46231</v>
-      </c>
-      <c r="F182" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="G182" s="7" t="s">
-        <v>1076</v>
-      </c>
-    </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A183" s="4"/>
-      <c r="B183" s="5"/>
-      <c r="C183" s="5"/>
-      <c r="D183" s="5"/>
-      <c r="E183" s="6"/>
-      <c r="F183" s="5"/>
-      <c r="G183" s="7"/>
-    </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A184" s="4"/>
-      <c r="B184" s="5"/>
-      <c r="C184" s="5"/>
-      <c r="D184" s="5"/>
-      <c r="E184" s="6"/>
-      <c r="F184" s="5"/>
-      <c r="G184" s="7"/>
-    </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A185" s="4"/>
-      <c r="B185" s="5"/>
-      <c r="C185" s="5"/>
-      <c r="D185" s="5"/>
-      <c r="E185" s="6"/>
-      <c r="F185" s="5"/>
-      <c r="G185" s="7"/>
-    </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A186" s="4"/>
-      <c r="B186" s="5"/>
-      <c r="C186" s="5"/>
-      <c r="D186" s="5"/>
-      <c r="E186" s="6"/>
-      <c r="F186" s="5"/>
-      <c r="G186" s="7"/>
-    </row>
-    <row r="187" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A187" s="4"/>
-      <c r="B187" s="5"/>
-      <c r="C187" s="5"/>
-      <c r="D187" s="5"/>
-      <c r="E187" s="6"/>
-      <c r="F187" s="5"/>
-      <c r="G187" s="7"/>
-    </row>
-    <row r="188" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A188" s="8">
-        <f>SUBTOTAL(9,A2:A187)</f>
-        <v>274000</v>
+      <c r="A159" s="4"/>
+      <c r="B159" s="5"/>
+      <c r="C159" s="5"/>
+      <c r="D159" s="5"/>
+      <c r="E159" s="6"/>
+      <c r="F159" s="5"/>
+      <c r="G159" s="7"/>
+    </row>
+    <row r="160" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A160" s="4"/>
+      <c r="B160" s="5"/>
+      <c r="C160" s="5"/>
+      <c r="D160" s="5"/>
+      <c r="E160" s="6"/>
+      <c r="F160" s="5"/>
+      <c r="G160" s="7"/>
+    </row>
+    <row r="161" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A161" s="8">
+        <f>SUBTOTAL(9,A2:A160)</f>
+        <v>378900</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G159" xr:uid="{19B3CF06-6FB5-4DC6-B5B9-AD7C386B2CA3}">
+  <autoFilter ref="A1:G125" xr:uid="{19B3CF06-6FB5-4DC6-B5B9-AD7C386B2CA3}">
     <filterColumn colId="6">
       <filters>
         <filter val="PENDIENTE"/>

</xml_diff>